<commit_message>
checkpoint : before adding productin explore.tsx
</commit_message>
<xml_diff>
--- a/docs/TimeSheet.xlsx
+++ b/docs/TimeSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\workplace\lsevin\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6F01704-1BC0-419C-938E-9F9A5EE1C3CB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67794594-9F65-4500-ABBB-0127FA8E496F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3C67C6F1-DCD5-4F32-8E1E-2D0F4630EB6C}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="181">
   <si>
     <t xml:space="preserve">عنوان </t>
   </si>
@@ -571,6 +571,9 @@
   </si>
   <si>
     <t>Important Information</t>
+  </si>
+  <si>
+    <t>انجام شده</t>
   </si>
 </sst>
 </file>
@@ -956,987 +959,1027 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5151749-D98A-4C10-BD15-AFBB1EC4BCB9}">
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:F164"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="43.140625" customWidth="1"/>
-    <col min="3" max="3" width="25.140625" customWidth="1"/>
-    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7"/>
+      <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>180</v>
+      </c>
+      <c r="C8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>180</v>
+      </c>
+      <c r="C9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>180</v>
+      </c>
+      <c r="C13" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C14" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="16" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>180</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C24" t="s">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D24" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C25" t="s">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C26" t="s">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D26" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C27" t="s">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D27" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+    <row r="28" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="E28" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="32" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+    <row r="32" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="35" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
+    <row r="35" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C36" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B38" t="s">
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B39" t="s">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
+    <row r="40" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B41" t="s">
+    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B43" t="s">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C43" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B44" s="1" t="s">
+    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C44" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B45" t="s">
+    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C45" t="s">
         <v>146</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="46" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
+    <row r="46" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="E46" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B47" t="s">
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C47" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C48" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B49" t="s">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C49" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="51" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
+    <row r="51" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D51" s="1" t="s">
+      <c r="E51" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B52" t="s">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C52" t="s">
         <v>47</v>
       </c>
-      <c r="D52">
+      <c r="E52">
         <v>0.5</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C53" t="s">
+    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
         <v>48</v>
       </c>
-      <c r="D53">
+      <c r="E53">
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C54" t="s">
+    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D54" t="s">
         <v>49</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B55" t="s">
+    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C55" t="s">
         <v>50</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B56" t="s">
+    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C56" t="s">
         <v>51</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B57" t="s">
+    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C57" t="s">
         <v>52</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B58" t="s">
+    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C58" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B59" t="s">
+    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C59" t="s">
         <v>54</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B60" t="s">
+    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C60" t="s">
         <v>55</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B61" t="s">
+    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C61" t="s">
         <v>56</v>
       </c>
-      <c r="D61" t="s">
+      <c r="E61" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="62" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="s">
+    <row r="62" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D62" s="1" t="s">
+      <c r="E62" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B63" t="s">
+    <row r="63" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C63" t="s">
         <v>89</v>
       </c>
-      <c r="D63" t="s">
+      <c r="E63" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B64" t="s">
+    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C64" t="s">
         <v>57</v>
       </c>
-      <c r="D64" t="s">
+      <c r="E64" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B65" t="s">
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C65" t="s">
         <v>88</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="67" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="s">
+    <row r="67" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B67" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="70" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="s">
+    <row r="70" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B70" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D70" s="1" t="s">
+      <c r="E70" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B71" t="s">
+    <row r="71" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C71" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C72" t="s">
+    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D72" t="s">
         <v>59</v>
       </c>
-      <c r="D72" t="s">
+      <c r="E72" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C73" t="s">
+    <row r="73" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D73" t="s">
         <v>60</v>
       </c>
-      <c r="D73" t="s">
+      <c r="E73" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C74" t="s">
+    <row r="74" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D74" t="s">
         <v>61</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E74" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C75" t="s">
+    <row r="75" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D75" t="s">
         <v>62</v>
       </c>
-      <c r="D75" t="s">
+      <c r="E75" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C76" t="s">
+    <row r="76" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D76" t="s">
         <v>63</v>
       </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C77" t="s">
+    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D77" t="s">
         <v>92</v>
       </c>
-      <c r="D77" t="s">
+      <c r="E77" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C78" t="s">
+    <row r="78" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D78" t="s">
         <v>93</v>
       </c>
-      <c r="D78" t="s">
+      <c r="E78" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="1" t="s">
+    <row r="79" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B79" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D79" s="1" t="s">
+      <c r="E79" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B80" t="s">
+    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C80" t="s">
         <v>64</v>
       </c>
-      <c r="D80" t="s">
+      <c r="E80" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="1" t="s">
+    <row r="82" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D82" s="1" t="s">
+      <c r="E82" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B83" t="s">
+    <row r="83" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C83" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B84" t="s">
+    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C84" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C85" t="s">
+    <row r="85" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D85" t="s">
         <v>66</v>
       </c>
-      <c r="D85" t="s">
+      <c r="E85" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C86" t="s">
+    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D86" t="s">
         <v>67</v>
       </c>
-      <c r="D86" t="s">
+      <c r="E86" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B87" t="s">
+    <row r="87" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C87" t="s">
         <v>95</v>
       </c>
-      <c r="D87" t="s">
+      <c r="E87" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B88" t="s">
+    <row r="88" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C88" t="s">
         <v>94</v>
       </c>
-      <c r="D88" t="s">
+      <c r="E88" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="1" t="s">
+    <row r="89" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B89" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D89" s="1" t="s">
+      <c r="E89" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B90" t="s">
+    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C90" t="s">
         <v>68</v>
       </c>
-      <c r="D90" t="s">
+      <c r="E90" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B91" t="s">
+    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C91" t="s">
         <v>69</v>
       </c>
-      <c r="D91" t="s">
+      <c r="E91" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B92" t="s">
+    <row r="92" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C92" t="s">
         <v>70</v>
       </c>
-      <c r="D92" t="s">
+      <c r="E92" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B93" t="s">
+    <row r="93" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C93" t="s">
         <v>71</v>
       </c>
-      <c r="D93" t="s">
+      <c r="E93" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B94" t="s">
+    <row r="94" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C94" t="s">
         <v>72</v>
       </c>
-      <c r="D94" t="s">
+      <c r="E94" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B95" t="s">
+    <row r="95" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C95" t="s">
         <v>73</v>
       </c>
-      <c r="D95" t="s">
+      <c r="E95" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B96" t="s">
+    <row r="96" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C96" t="s">
         <v>74</v>
       </c>
-      <c r="D96" t="s">
+      <c r="E96" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C97" t="s">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D97" t="s">
         <v>75</v>
       </c>
-      <c r="D97" t="s">
+      <c r="E97" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C98" t="s">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D98" t="s">
         <v>76</v>
       </c>
-      <c r="D98" t="s">
+      <c r="E98" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C99" t="s">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D99" t="s">
         <v>77</v>
       </c>
-      <c r="D99" t="s">
+      <c r="E99" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C100" t="s">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D100" t="s">
         <v>78</v>
       </c>
-      <c r="D100" t="s">
+      <c r="E100" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C101" t="s">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D101" t="s">
         <v>79</v>
       </c>
-      <c r="D101" t="s">
+      <c r="E101" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C102" t="s">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D102" t="s">
         <v>80</v>
       </c>
-      <c r="D102" t="s">
+      <c r="E102" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C103" t="s">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D103" t="s">
         <v>81</v>
       </c>
-      <c r="D103" t="s">
+      <c r="E103" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B104" t="s">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C104" t="s">
         <v>82</v>
       </c>
-      <c r="D104" t="s">
+      <c r="E104" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C105" t="s">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D105" t="s">
         <v>83</v>
       </c>
-      <c r="D105" t="s">
+      <c r="E105" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C106" t="s">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D106" t="s">
         <v>24</v>
       </c>
-      <c r="D106" t="s">
+      <c r="E106" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B107" t="s">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C107" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B108" t="s">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C108" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="109" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="1" t="s">
+    <row r="109" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B109" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B109" s="1" t="s">
+      <c r="C109" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D109" s="1" t="s">
+      <c r="E109" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B110" t="s">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>180</v>
+      </c>
+      <c r="C110" t="s">
         <v>84</v>
       </c>
-      <c r="D110" t="s">
+      <c r="E110" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B111" t="s">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>180</v>
+      </c>
+      <c r="C111" t="s">
         <v>85</v>
       </c>
-      <c r="D111" t="s">
+      <c r="E111" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B112" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B113" t="s">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C113" t="s">
         <v>103</v>
       </c>
-      <c r="D113" t="s">
+      <c r="E113" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="115" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="3" t="s">
+    <row r="115" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B115" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B115" s="3" t="s">
+      <c r="C115" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="D115" s="3" t="s">
+      <c r="E115" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="116" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B116" s="1" t="s">
+    <row r="116" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C116" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B117" t="s">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C117" t="s">
         <v>170</v>
       </c>
-      <c r="D117" t="s">
+      <c r="E117" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B118" t="s">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>180</v>
+      </c>
+      <c r="C118" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B119" t="s">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>180</v>
+      </c>
+      <c r="C119" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="120" spans="1:5" ht="24" x14ac:dyDescent="0.25">
-      <c r="B120" t="s">
+    <row r="120" spans="1:6" ht="24" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>180</v>
+      </c>
+      <c r="C120" t="s">
         <v>172</v>
       </c>
-      <c r="C120" s="4" t="s">
+      <c r="D120" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="D120" s="5" t="s">
+      <c r="E120" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="E120" s="6" t="s">
+      <c r="F120" s="6" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B121" t="s">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>180</v>
+      </c>
+      <c r="C121" t="s">
         <v>173</v>
       </c>
-      <c r="C121" s="6" t="s">
+      <c r="D121" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="D121" s="4" t="s">
+      <c r="E121" s="4" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B122" t="s">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>180</v>
+      </c>
+      <c r="C122" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B123" t="s">
         <v>123</v>
       </c>
-      <c r="B123" t="s">
+      <c r="C123" t="s">
         <v>138</v>
       </c>
-      <c r="C123" t="s">
+      <c r="D123" t="s">
         <v>139</v>
       </c>
-      <c r="D123" t="s">
+      <c r="E123" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C124" t="s">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D124" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
         <v>124</v>
       </c>
-      <c r="B125" t="s">
+      <c r="C125" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B126" t="s">
         <v>125</v>
       </c>
-      <c r="B126" s="2">
+      <c r="C126" s="2">
         <v>0.03</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B127" t="s">
         <v>126</v>
       </c>
-      <c r="B127" s="2">
+      <c r="C127" s="2">
         <v>0.02</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B128" t="s">
         <v>128</v>
       </c>
-      <c r="B128" s="2">
+      <c r="C128" s="2">
         <v>0.1</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
+    <row r="129" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B129" t="s">
         <v>129</v>
       </c>
-      <c r="B129" t="s">
+      <c r="C129" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
+    <row r="130" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B130" t="s">
         <v>131</v>
       </c>
-      <c r="B130" t="s">
+      <c r="C130" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B131" t="s">
+    <row r="131" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C131" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
+    <row r="132" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B132" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
+    <row r="133" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B133" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
+    <row r="134" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B134" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
+    <row r="135" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B135" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B137" t="s">
+    <row r="137" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C137" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B138" t="s">
+    <row r="138" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C138" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B139" t="s">
+    <row r="139" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C139" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B140" t="s">
+    <row r="140" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C140" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B141" t="s">
+    <row r="141" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C141" t="s">
         <v>150</v>
       </c>
-      <c r="C141" t="s">
+      <c r="D141" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C142" t="s">
+    <row r="142" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D142" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C143" t="s">
+    <row r="143" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D143" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C144" t="s">
+    <row r="144" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D144" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="145" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C145" t="s">
+    <row r="145" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D145" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="146" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C146" t="s">
+    <row r="146" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D146" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="147" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C147" t="s">
+    <row r="147" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D147" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="148" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C148" t="s">
+    <row r="148" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D148" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="149" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C149" t="s">
+    <row r="149" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D149" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="150" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B150" t="s">
+    <row r="150" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C150" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="151" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B151" t="s">
+    <row r="151" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C151" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="154" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B154" t="s">
+    <row r="154" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C154" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="155" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B155" t="s">
+    <row r="155" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C155" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="156" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B156" t="s">
+    <row r="156" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C156" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="157" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B157" t="s">
+    <row r="157" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C157" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B163" t="s">
+    <row r="163" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C163" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B164" t="s">
+    <row r="164" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C164" t="s">
         <v>116</v>
       </c>
     </row>

</xml_diff>

<commit_message>
checkpoint: before map-discovery edit
</commit_message>
<xml_diff>
--- a/docs/TimeSheet.xlsx
+++ b/docs/TimeSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\workplace\lsevin\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67794594-9F65-4500-ABBB-0127FA8E496F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C426C7AD-7F9F-40B0-8A48-370930D1B27C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3C67C6F1-DCD5-4F32-8E1E-2D0F4630EB6C}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="183">
   <si>
     <t xml:space="preserve">عنوان </t>
   </si>
@@ -574,6 +574,12 @@
   </si>
   <si>
     <t>انجام شده</t>
+  </si>
+  <si>
+    <t xml:space="preserve">تصویر برای category ها در ادمین و نمایش در صفحه </t>
+  </si>
+  <si>
+    <t>اصلاح دیتای view all برای cateogory ها</t>
   </si>
 </sst>
 </file>
@@ -959,7 +965,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5151749-D98A-4C10-BD15-AFBB1EC4BCB9}">
-  <dimension ref="A1:F164"/>
+  <dimension ref="A1:F165"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.42578125" customWidth="1"/>
@@ -1158,12 +1164,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="35" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
         <v>12</v>
       </c>
@@ -1171,52 +1177,52 @@
         <v>142</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C37" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C39" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C41" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C43" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C44" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C45" t="s">
         <v>146</v>
       </c>
@@ -1224,7 +1230,10 @@
         <v>101</v>
       </c>
     </row>
-    <row r="46" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>180</v>
+      </c>
       <c r="B46" s="1" t="s">
         <v>16</v>
       </c>
@@ -1232,167 +1241,181 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>180</v>
+      </c>
       <c r="C47" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>180</v>
+      </c>
       <c r="C48" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>180</v>
+      </c>
       <c r="C49" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="51" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="1" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C50" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>180</v>
+      </c>
+      <c r="C51" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E51" s="1" t="s">
+      <c r="E52" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C52" t="s">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C53" t="s">
         <v>47</v>
       </c>
-      <c r="E52">
+      <c r="E53">
         <v>0.5</v>
       </c>
     </row>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D53" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D54" t="s">
         <v>48</v>
       </c>
-      <c r="E53">
+      <c r="E54">
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D54" t="s">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D55" t="s">
         <v>49</v>
       </c>
-      <c r="E54" t="s">
+      <c r="E55" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C55" t="s">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C56" t="s">
         <v>50</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E56" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C56" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C57" t="s">
         <v>51</v>
-      </c>
-      <c r="E56" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C57" t="s">
-        <v>52</v>
       </c>
       <c r="E57" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C58" t="s">
+        <v>52</v>
+      </c>
+      <c r="E58" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C59" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C59" t="s">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C60" t="s">
         <v>54</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E60" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C60" t="s">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C61" t="s">
         <v>55</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E61" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C61" t="s">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C62" t="s">
         <v>56</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E62" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="62" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="1" t="s">
+    <row r="63" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B63" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E62" s="1" t="s">
+      <c r="E63" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="63" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C63" t="s">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C64" t="s">
         <v>89</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E64" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C64" t="s">
-        <v>57</v>
-      </c>
-      <c r="E64" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
+        <v>57</v>
+      </c>
+      <c r="E65" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C66" t="s">
         <v>88</v>
       </c>
-      <c r="E65" t="s">
+      <c r="E66" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="67" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="1" t="s">
+    <row r="68" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B68" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="70" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="1" t="s">
+    <row r="71" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B71" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E70" s="1" t="s">
+      <c r="E71" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="71" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C71" t="s">
+    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C72" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D72" t="s">
-        <v>59</v>
-      </c>
-      <c r="E72" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D73" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E73" t="s">
         <v>87</v>
@@ -1400,15 +1423,15 @@
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D74" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E74" t="s">
-        <v>3</v>
+        <v>87</v>
       </c>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D75" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E75" t="s">
         <v>3</v>
@@ -1416,81 +1439,81 @@
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D76" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E76" t="s">
-        <v>87</v>
+        <v>3</v>
       </c>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D77" t="s">
-        <v>92</v>
+        <v>63</v>
       </c>
       <c r="E77" t="s">
-        <v>3</v>
+        <v>87</v>
       </c>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D78" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E78" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="1" t="s">
+    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D79" t="s">
+        <v>93</v>
+      </c>
+      <c r="E79" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B80" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E79" s="1" t="s">
+      <c r="E80" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C80" t="s">
+    <row r="81" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C81" t="s">
         <v>64</v>
       </c>
-      <c r="E80" t="s">
+      <c r="E81" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="1" t="s">
+    <row r="83" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="E83" s="1" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C83" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="84" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C84" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="85" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C85" t="s">
         <v>86</v>
-      </c>
-    </row>
-    <row r="85" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D85" t="s">
-        <v>66</v>
-      </c>
-      <c r="E85" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="86" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D86" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E86" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="87" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C87" t="s">
-        <v>95</v>
+      <c r="D87" t="s">
+        <v>67</v>
       </c>
       <c r="E87" t="s">
         <v>3</v>
@@ -1498,39 +1521,39 @@
     </row>
     <row r="88" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C88" t="s">
+        <v>95</v>
+      </c>
+      <c r="E88" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C89" t="s">
         <v>94</v>
       </c>
-      <c r="E88" t="s">
+      <c r="E89" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B89" s="1" t="s">
+    <row r="90" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B90" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E89" s="1" t="s">
+      <c r="E90" s="1" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C90" t="s">
-        <v>68</v>
-      </c>
-      <c r="E90" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="91" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C91" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E91" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
     </row>
     <row r="92" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C92" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E92" t="s">
         <v>10</v>
@@ -1538,39 +1561,39 @@
     </row>
     <row r="93" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C93" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E93" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
     </row>
     <row r="94" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C94" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E94" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="95" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C95" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E95" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
     </row>
     <row r="96" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C96" t="s">
+        <v>73</v>
+      </c>
+      <c r="E96" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C97" t="s">
         <v>74</v>
-      </c>
-      <c r="E96" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D97" t="s">
-        <v>75</v>
       </c>
       <c r="E97" t="s">
         <v>100</v>
@@ -1578,7 +1601,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D98" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E98" t="s">
         <v>100</v>
@@ -1586,7 +1609,7 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D99" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E99" t="s">
         <v>100</v>
@@ -1594,7 +1617,7 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D100" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E100" t="s">
         <v>100</v>
@@ -1602,7 +1625,7 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D101" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E101" t="s">
         <v>100</v>
@@ -1610,7 +1633,7 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D102" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E102" t="s">
         <v>100</v>
@@ -1618,23 +1641,23 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D103" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E103" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C104" t="s">
-        <v>82</v>
+      <c r="D104" t="s">
+        <v>81</v>
       </c>
       <c r="E104" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D105" t="s">
-        <v>83</v>
+      <c r="C105" t="s">
+        <v>82</v>
       </c>
       <c r="E105" t="s">
         <v>100</v>
@@ -1642,42 +1665,39 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D106" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E106" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C107" t="s">
-        <v>109</v>
+      <c r="D107" t="s">
+        <v>24</v>
+      </c>
+      <c r="E107" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C108" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C109" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="109" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B109" s="1" t="s">
+    <row r="110" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B110" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C109" s="1" t="s">
+      <c r="C110" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="E109" s="1" t="s">
+      <c r="E110" s="1" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>180</v>
-      </c>
-      <c r="C110" t="s">
-        <v>84</v>
-      </c>
-      <c r="E110" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
@@ -1685,55 +1705,58 @@
         <v>180</v>
       </c>
       <c r="C111" t="s">
+        <v>84</v>
+      </c>
+      <c r="E111" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>180</v>
+      </c>
+      <c r="C112" t="s">
         <v>85</v>
       </c>
-      <c r="E111" t="s">
+      <c r="E112" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B112" t="s">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B113" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C113" t="s">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C114" t="s">
         <v>103</v>
       </c>
-      <c r="E113" t="s">
+      <c r="E114" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="115" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B115" s="3" t="s">
+    <row r="116" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B116" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C115" s="3" t="s">
+      <c r="C116" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E115" s="3" t="s">
+      <c r="E116" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="116" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C116" s="1" t="s">
+    <row r="117" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C117" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C117" t="s">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C118" t="s">
         <v>170</v>
       </c>
-      <c r="E117" t="s">
+      <c r="E118" t="s">
         <v>169</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>180</v>
-      </c>
-      <c r="C118" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
@@ -1741,38 +1764,32 @@
         <v>180</v>
       </c>
       <c r="C119" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" ht="24" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>180</v>
       </c>
       <c r="C120" t="s">
-        <v>172</v>
-      </c>
-      <c r="D120" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="E120" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="F120" s="6" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="24" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>180</v>
       </c>
       <c r="C121" t="s">
-        <v>173</v>
-      </c>
-      <c r="D121" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="E121" s="4" t="s">
-        <v>177</v>
+        <v>172</v>
+      </c>
+      <c r="D121" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="E121" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="F121" s="6" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
@@ -1780,206 +1797,220 @@
         <v>180</v>
       </c>
       <c r="C122" t="s">
+        <v>173</v>
+      </c>
+      <c r="D122" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="E122" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>180</v>
+      </c>
+      <c r="C123" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B123" t="s">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B124" t="s">
         <v>123</v>
       </c>
-      <c r="C123" t="s">
+      <c r="C124" t="s">
         <v>138</v>
       </c>
-      <c r="D123" t="s">
+      <c r="D124" t="s">
         <v>139</v>
       </c>
-      <c r="E123" t="s">
+      <c r="E124" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D124" t="s">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D125" t="s">
         <v>140</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B125" t="s">
-        <v>124</v>
-      </c>
-      <c r="C125" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B126" t="s">
-        <v>125</v>
-      </c>
-      <c r="C126" s="2">
-        <v>0.03</v>
+        <v>124</v>
+      </c>
+      <c r="C126" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B127" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C127" s="2">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B128" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C128" s="2">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="129" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B129" t="s">
-        <v>129</v>
-      </c>
-      <c r="C129" t="s">
-        <v>130</v>
+        <v>128</v>
+      </c>
+      <c r="C129" s="2">
+        <v>0.1</v>
       </c>
     </row>
     <row r="130" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B130" t="s">
+        <v>129</v>
+      </c>
+      <c r="C130" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="131" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B131" t="s">
         <v>131</v>
       </c>
-      <c r="C130" t="s">
+      <c r="C131" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="131" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C131" t="s">
+    <row r="132" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C132" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="132" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B132" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="133" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B133" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="134" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="135" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B135" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="136" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B136" t="s">
         <v>137</v>
-      </c>
-    </row>
-    <row r="137" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C137" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="138" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C138" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="139" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C139" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
     </row>
     <row r="140" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C140" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
     </row>
     <row r="141" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C141" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="142" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C142" t="s">
         <v>150</v>
       </c>
-      <c r="D141" t="s">
+      <c r="D142" t="s">
         <v>151</v>
-      </c>
-    </row>
-    <row r="142" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D142" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="143" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D143" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="144" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D144" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="145" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D145" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="146" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D146" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="147" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D147" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="148" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D148" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="149" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D149" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="150" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D150" t="s">
         <v>159</v>
-      </c>
-    </row>
-    <row r="150" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C150" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="151" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C151" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="152" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C152" t="s">
         <v>161</v>
-      </c>
-    </row>
-    <row r="154" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C154" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="155" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C155" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="156" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C156" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="157" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C157" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="158" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C158" t="s">
         <v>120</v>
-      </c>
-    </row>
-    <row r="163" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C163" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="164" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C164" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="165" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C165" t="s">
         <v>116</v>
       </c>
     </row>

</xml_diff>

<commit_message>
checkpoint: rewards, coupans , wallet
</commit_message>
<xml_diff>
--- a/docs/TimeSheet.xlsx
+++ b/docs/TimeSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\workplace\lsevin\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C426C7AD-7F9F-40B0-8A48-370930D1B27C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C1196B-1CD4-45C8-8E76-5FE389E0519C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3C67C6F1-DCD5-4F32-8E1E-2D0F4630EB6C}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="184">
   <si>
     <t xml:space="preserve">عنوان </t>
   </si>
@@ -580,6 +580,9 @@
   </si>
   <si>
     <t>اصلاح دیتای view all برای cateogory ها</t>
+  </si>
+  <si>
+    <t>nearby - map</t>
   </si>
 </sst>
 </file>
@@ -965,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5151749-D98A-4C10-BD15-AFBB1EC4BCB9}">
-  <dimension ref="A1:F165"/>
+  <dimension ref="A1:F166"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.42578125" customWidth="1"/>
@@ -1009,20 +1012,20 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>180</v>
+      </c>
       <c r="B7" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8"/>
+      <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>180</v>
-      </c>
-      <c r="C8" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1030,30 +1033,30 @@
         <v>180</v>
       </c>
       <c r="C9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>180</v>
+      </c>
+      <c r="C10" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C10" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
         <v>105</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>180</v>
-      </c>
-      <c r="C13" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -1061,192 +1064,210 @@
         <v>180</v>
       </c>
       <c r="C14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>180</v>
+      </c>
+      <c r="C15" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C15" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>180</v>
-      </c>
-      <c r="B16" s="1" t="s">
+    <row r="17" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>180</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C17" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C18" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C19" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="1" t="s">
+    <row r="22" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>180</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C22" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>180</v>
+      </c>
+      <c r="C23" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C23" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>180</v>
+      </c>
+      <c r="C24" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D24" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D25" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D26" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D26" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D27" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D27" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="1" t="s">
+    <row r="29" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>180</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E29" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C29" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C30" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C31" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="32" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="1" t="s">
+    <row r="33" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="E33" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C33" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C34" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="1" t="s">
+    <row r="36" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="E36" s="1" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C36" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C37" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
-        <v>143</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C39" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="1" t="s">
+    <row r="41" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C41" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C42" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="1" t="s">
+    <row r="43" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C43" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>180</v>
+      </c>
+      <c r="C44" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C44" s="1" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>180</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C45" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C46" t="s">
         <v>146</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E46" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="46" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>180</v>
-      </c>
-      <c r="B46" s="1" t="s">
+    <row r="47" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>180</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E47" s="1" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>180</v>
-      </c>
-      <c r="C47" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -1254,7 +1275,7 @@
         <v>180</v>
       </c>
       <c r="C48" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -1262,73 +1283,73 @@
         <v>180</v>
       </c>
       <c r="C49" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>180</v>
+      </c>
+      <c r="C50" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C50" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C51" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>180</v>
-      </c>
-      <c r="C51" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>180</v>
+      </c>
+      <c r="C52" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="52" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="1" t="s">
+    <row r="53" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E53" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C53" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C54" t="s">
         <v>47</v>
       </c>
-      <c r="E53">
+      <c r="E54">
         <v>0.5</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D54" t="s">
-        <v>48</v>
-      </c>
-      <c r="E54">
-        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D55" t="s">
+        <v>48</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D56" t="s">
         <v>49</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E56" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C56" t="s">
-        <v>50</v>
-      </c>
-      <c r="E56" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C57" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E57" t="s">
-        <v>87</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C58" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E58" t="s">
         <v>87</v>
@@ -1336,192 +1357,204 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C59" t="s">
-        <v>53</v>
+        <v>52</v>
+      </c>
+      <c r="E59" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C60" t="s">
-        <v>54</v>
-      </c>
-      <c r="E60" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C61" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E61" t="s">
-        <v>147</v>
+        <v>13</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C62" t="s">
+        <v>55</v>
+      </c>
+      <c r="E62" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C63" t="s">
         <v>56</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E63" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="63" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="1" t="s">
+    <row r="64" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B64" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E63" s="1" t="s">
+      <c r="E64" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C64" t="s">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>180</v>
+      </c>
+      <c r="C65" t="s">
         <v>89</v>
       </c>
-      <c r="E64" t="s">
+      <c r="E65" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C65" t="s">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C66" t="s">
         <v>57</v>
       </c>
-      <c r="E65" t="s">
+      <c r="E66" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C66" t="s">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>180</v>
+      </c>
+      <c r="C67" t="s">
         <v>88</v>
       </c>
-      <c r="E66" t="s">
+      <c r="E67" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="68" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="1" t="s">
+    <row r="69" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>180</v>
+      </c>
+      <c r="B69" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="71" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="1" t="s">
+    <row r="72" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B72" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E71" s="1" t="s">
+      <c r="E72" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C72" t="s">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>180</v>
+      </c>
+      <c r="C73" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="73" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D73" t="s">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D74" t="s">
         <v>59</v>
-      </c>
-      <c r="E73" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="74" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D74" t="s">
-        <v>60</v>
       </c>
       <c r="E74" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="75" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D75" t="s">
+        <v>60</v>
+      </c>
+      <c r="E75" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D76" t="s">
         <v>61</v>
-      </c>
-      <c r="E75" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="76" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D76" t="s">
-        <v>62</v>
       </c>
       <c r="E76" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D77" t="s">
+        <v>62</v>
+      </c>
+      <c r="E77" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D78" t="s">
         <v>63</v>
       </c>
-      <c r="E77" t="s">
+      <c r="E78" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="78" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D78" t="s">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D79" t="s">
         <v>92</v>
-      </c>
-      <c r="E78" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D79" t="s">
-        <v>93</v>
       </c>
       <c r="E79" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B80" s="1" t="s">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D80" t="s">
+        <v>93</v>
+      </c>
+      <c r="E80" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="81" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B81" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E80" s="1" t="s">
+      <c r="E81" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C81" t="s">
+    <row r="82" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C82" t="s">
         <v>64</v>
       </c>
-      <c r="E81" t="s">
+      <c r="E82" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="1" t="s">
+    <row r="84" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E83" s="1" t="s">
+      <c r="E84" s="1" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C84" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="85" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C85" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C86" t="s">
         <v>86</v>
-      </c>
-    </row>
-    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D86" t="s">
-        <v>66</v>
-      </c>
-      <c r="E86" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="87" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D87" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E87" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="88" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C88" t="s">
-        <v>95</v>
+      <c r="D88" t="s">
+        <v>67</v>
       </c>
       <c r="E88" t="s">
         <v>3</v>
@@ -1529,39 +1562,39 @@
     </row>
     <row r="89" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C89" t="s">
+        <v>95</v>
+      </c>
+      <c r="E89" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C90" t="s">
         <v>94</v>
       </c>
-      <c r="E89" t="s">
+      <c r="E90" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="90" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B90" s="1" t="s">
+    <row r="91" spans="2:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B91" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E90" s="1" t="s">
+      <c r="E91" s="1" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C91" t="s">
-        <v>68</v>
-      </c>
-      <c r="E91" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="92" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C92" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E92" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
     </row>
     <row r="93" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C93" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E93" t="s">
         <v>10</v>
@@ -1569,39 +1602,39 @@
     </row>
     <row r="94" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C94" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E94" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
     </row>
     <row r="95" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C95" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E95" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="96" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C96" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E96" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C97" t="s">
+        <v>73</v>
+      </c>
+      <c r="E97" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C98" t="s">
         <v>74</v>
-      </c>
-      <c r="E97" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D98" t="s">
-        <v>75</v>
       </c>
       <c r="E98" t="s">
         <v>100</v>
@@ -1609,7 +1642,7 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D99" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E99" t="s">
         <v>100</v>
@@ -1617,7 +1650,7 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D100" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E100" t="s">
         <v>100</v>
@@ -1625,7 +1658,7 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D101" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E101" t="s">
         <v>100</v>
@@ -1633,7 +1666,7 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D102" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E102" t="s">
         <v>100</v>
@@ -1641,7 +1674,7 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D103" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E103" t="s">
         <v>100</v>
@@ -1649,23 +1682,23 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D104" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E104" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C105" t="s">
-        <v>82</v>
+      <c r="D105" t="s">
+        <v>81</v>
       </c>
       <c r="E105" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D106" t="s">
-        <v>83</v>
+      <c r="C106" t="s">
+        <v>82</v>
       </c>
       <c r="E106" t="s">
         <v>100</v>
@@ -1673,42 +1706,39 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D107" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E107" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C108" t="s">
-        <v>109</v>
+      <c r="D108" t="s">
+        <v>24</v>
+      </c>
+      <c r="E108" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C109" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C110" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="110" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B110" s="1" t="s">
+    <row r="111" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B111" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C110" s="1" t="s">
+      <c r="C111" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="E110" s="1" t="s">
+      <c r="E111" s="1" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>180</v>
-      </c>
-      <c r="C111" t="s">
-        <v>84</v>
-      </c>
-      <c r="E111" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
@@ -1716,55 +1746,58 @@
         <v>180</v>
       </c>
       <c r="C112" t="s">
+        <v>84</v>
+      </c>
+      <c r="E112" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>180</v>
+      </c>
+      <c r="C113" t="s">
         <v>85</v>
       </c>
-      <c r="E112" t="s">
+      <c r="E113" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B113" t="s">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B114" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C114" t="s">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C115" t="s">
         <v>103</v>
       </c>
-      <c r="E114" t="s">
+      <c r="E115" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="116" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B116" s="3" t="s">
+    <row r="117" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B117" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C116" s="3" t="s">
+      <c r="C117" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E116" s="3" t="s">
+      <c r="E117" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="117" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C117" s="1" t="s">
+    <row r="118" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C118" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C118" t="s">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C119" t="s">
         <v>170</v>
       </c>
-      <c r="E118" t="s">
+      <c r="E119" t="s">
         <v>169</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>180</v>
-      </c>
-      <c r="C119" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
@@ -1772,38 +1805,32 @@
         <v>180</v>
       </c>
       <c r="C120" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>180</v>
+      </c>
+      <c r="C121" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="121" spans="1:6" ht="24" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>180</v>
-      </c>
-      <c r="C121" t="s">
+    <row r="122" spans="1:6" ht="24" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>180</v>
+      </c>
+      <c r="C122" t="s">
         <v>172</v>
       </c>
-      <c r="D121" s="4" t="s">
+      <c r="D122" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="E121" s="5" t="s">
+      <c r="E122" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="F121" s="6" t="s">
+      <c r="F122" s="6" t="s">
         <v>178</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>180</v>
-      </c>
-      <c r="C122" t="s">
-        <v>173</v>
-      </c>
-      <c r="D122" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="E122" s="4" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
@@ -1811,206 +1838,223 @@
         <v>180</v>
       </c>
       <c r="C123" t="s">
+        <v>173</v>
+      </c>
+      <c r="D123" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="E123" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>180</v>
+      </c>
+      <c r="C124" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B124" t="s">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>180</v>
+      </c>
+      <c r="B125" t="s">
         <v>123</v>
       </c>
-      <c r="C124" t="s">
+      <c r="C125" t="s">
         <v>138</v>
       </c>
-      <c r="D124" t="s">
+      <c r="D125" t="s">
         <v>139</v>
       </c>
-      <c r="E124" t="s">
+      <c r="E125" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D125" t="s">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D126" t="s">
         <v>140</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B126" t="s">
-        <v>124</v>
-      </c>
-      <c r="C126" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B127" t="s">
-        <v>125</v>
-      </c>
-      <c r="C127" s="2">
-        <v>0.03</v>
+        <v>124</v>
+      </c>
+      <c r="C127" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B128" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C128" s="2">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="129" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B129" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C129" s="2">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="130" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B130" t="s">
-        <v>129</v>
-      </c>
-      <c r="C130" t="s">
-        <v>130</v>
+        <v>128</v>
+      </c>
+      <c r="C130" s="2">
+        <v>0.1</v>
       </c>
     </row>
     <row r="131" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B131" t="s">
+        <v>129</v>
+      </c>
+      <c r="C131" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="132" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B132" t="s">
         <v>131</v>
       </c>
-      <c r="C131" t="s">
+      <c r="C132" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="132" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C132" t="s">
+    <row r="133" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C133" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="133" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B133" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="134" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="135" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B135" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="136" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B136" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="137" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B137" t="s">
         <v>137</v>
-      </c>
-    </row>
-    <row r="138" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C138" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="139" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C139" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="140" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C140" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
     </row>
     <row r="141" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C141" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
     </row>
     <row r="142" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C142" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="143" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C143" t="s">
         <v>150</v>
       </c>
-      <c r="D142" t="s">
+      <c r="D143" t="s">
         <v>151</v>
-      </c>
-    </row>
-    <row r="143" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D143" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="144" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D144" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="145" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D145" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="146" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D146" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="147" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D147" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="148" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D148" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="149" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D149" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="150" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D150" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="151" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D151" t="s">
         <v>159</v>
-      </c>
-    </row>
-    <row r="151" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C151" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="152" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C152" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="153" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C153" t="s">
         <v>161</v>
-      </c>
-    </row>
-    <row r="155" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C155" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="156" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C156" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="157" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C157" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="158" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C158" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="159" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C159" t="s">
         <v>120</v>
-      </c>
-    </row>
-    <row r="164" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C164" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="165" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C165" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="166" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C166" t="s">
         <v>116</v>
       </c>
     </row>

</xml_diff>

<commit_message>
before dynamic form new version
</commit_message>
<xml_diff>
--- a/docs/TimeSheet.xlsx
+++ b/docs/TimeSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\workplace\lsevin\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C1196B-1CD4-45C8-8E76-5FE389E0519C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8985940-BD07-404E-A835-4EBB28A52574}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3C67C6F1-DCD5-4F32-8E1E-2D0F4630EB6C}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="183">
   <si>
     <t xml:space="preserve">عنوان </t>
   </si>
@@ -412,9 +412,6 @@
   </si>
   <si>
     <t>دعوت</t>
-  </si>
-  <si>
-    <t>5%^</t>
   </si>
   <si>
     <t xml:space="preserve">جمع ثبت نام </t>
@@ -979,7 +976,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B1" t="s">
         <v>114</v>
@@ -1013,10 +1010,10 @@
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1030,7 +1027,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C9" t="s">
         <v>28</v>
@@ -1038,7 +1035,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C10" t="s">
         <v>29</v>
@@ -1061,7 +1058,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C14" t="s">
         <v>106</v>
@@ -1069,7 +1066,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C15" t="s">
         <v>107</v>
@@ -1082,7 +1079,7 @@
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>6</v>
@@ -1108,7 +1105,7 @@
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>8</v>
@@ -1119,7 +1116,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C23" t="s">
         <v>36</v>
@@ -1127,7 +1124,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C24" t="s">
         <v>37</v>
@@ -1155,7 +1152,7 @@
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>9</v>
@@ -1197,7 +1194,7 @@
         <v>12</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1212,7 +1209,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C39" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1237,23 +1234,23 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C44" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C46" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E46" t="s">
         <v>101</v>
@@ -1261,7 +1258,7 @@
     </row>
     <row r="47" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>16</v>
@@ -1272,7 +1269,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C48" t="s">
         <v>44</v>
@@ -1280,7 +1277,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C49" t="s">
         <v>45</v>
@@ -1288,7 +1285,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C50" t="s">
         <v>46</v>
@@ -1296,15 +1293,15 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C51" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>179</v>
+      </c>
+      <c r="C52" t="s">
         <v>180</v>
-      </c>
-      <c r="C52" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="53" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1381,7 +1378,7 @@
         <v>55</v>
       </c>
       <c r="E62" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -1389,7 +1386,7 @@
         <v>56</v>
       </c>
       <c r="E63" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1402,7 +1399,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C65" t="s">
         <v>89</v>
@@ -1421,7 +1418,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C67" t="s">
         <v>88</v>
@@ -1432,7 +1429,7 @@
     </row>
     <row r="69" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>19</v>
@@ -1448,7 +1445,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C73" t="s">
         <v>58</v>
@@ -1735,7 +1732,7 @@
         <v>25</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E111" s="1" t="s">
         <v>101</v>
@@ -1743,7 +1740,7 @@
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C112" t="s">
         <v>84</v>
@@ -1754,7 +1751,7 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C113" t="s">
         <v>85</v>
@@ -1781,7 +1778,7 @@
         <v>25</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E117" s="3" t="s">
         <v>101</v>
@@ -1789,100 +1786,100 @@
     </row>
     <row r="118" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C118" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C119" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E119" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C120" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C121" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="24" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C122" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D122" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E122" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="E122" s="5" t="s">
-        <v>175</v>
-      </c>
       <c r="F122" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C123" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D123" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="E123" s="4" t="s">
         <v>176</v>
-      </c>
-      <c r="E123" s="4" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C124" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B125" t="s">
         <v>123</v>
       </c>
       <c r="C125" t="s">
+        <v>137</v>
+      </c>
+      <c r="D125" t="s">
         <v>138</v>
       </c>
-      <c r="D125" t="s">
-        <v>139</v>
-      </c>
       <c r="E125" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D126" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B127" t="s">
         <v>124</v>
       </c>
-      <c r="C127" t="s">
-        <v>127</v>
+      <c r="C127" s="2">
+        <v>0.05</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
@@ -1903,7 +1900,7 @@
     </row>
     <row r="130" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B130" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C130" s="2">
         <v>0.1</v>
@@ -1911,121 +1908,121 @@
     </row>
     <row r="131" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B131" t="s">
+        <v>128</v>
+      </c>
+      <c r="C131" t="s">
         <v>129</v>
-      </c>
-      <c r="C131" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="132" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B132" t="s">
+        <v>130</v>
+      </c>
+      <c r="C132" t="s">
         <v>131</v>
-      </c>
-      <c r="C132" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="133" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C133" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="134" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="135" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B135" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="136" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B136" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="137" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B137" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="139" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C139" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="140" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C140" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="141" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C141" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="142" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C142" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="143" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C143" t="s">
+        <v>149</v>
+      </c>
+      <c r="D143" t="s">
         <v>150</v>
-      </c>
-      <c r="D143" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="144" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D144" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="145" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D145" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="146" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D146" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="147" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D147" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="148" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D148" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="149" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D149" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="150" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D150" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="151" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D151" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="152" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C152" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="153" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C153" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="156" spans="3:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
before admin panel changes
</commit_message>
<xml_diff>
--- a/docs/TimeSheet.xlsx
+++ b/docs/TimeSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\workplace\lsevin\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F3BC1DF-CB2A-4281-9E21-0BB46C173099}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC38802-6E75-467D-B0B8-4F16F51FFD84}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3C67C6F1-DCD5-4F32-8E1E-2D0F4630EB6C}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="192">
   <si>
     <t xml:space="preserve">عنوان </t>
   </si>
@@ -589,6 +589,24 @@
   </si>
   <si>
     <t>فرم ساز پیشرفته برای هر سرویس</t>
+  </si>
+  <si>
+    <t>ثبت در جدول customers در زمان ثبت نام</t>
+  </si>
+  <si>
+    <t>notifications</t>
+  </si>
+  <si>
+    <t>/medical-profile</t>
+  </si>
+  <si>
+    <t>/privacy-security/</t>
+  </si>
+  <si>
+    <t>settings</t>
+  </si>
+  <si>
+    <t>my bookings</t>
   </si>
 </sst>
 </file>
@@ -981,7 +999,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5151749-D98A-4C10-BD15-AFBB1EC4BCB9}">
-  <dimension ref="A1:F170"/>
+  <dimension ref="A1:F177"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.42578125" customWidth="1"/>
@@ -2086,29 +2104,74 @@
         <v>117</v>
       </c>
     </row>
-    <row r="161" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C161" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="162" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C162" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="163" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C163" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="169" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C169" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="170" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C170" t="s">
         <v>116</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B172" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>179</v>
+      </c>
+      <c r="B173" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>179</v>
+      </c>
+      <c r="B174" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>179</v>
+      </c>
+      <c r="B175" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>179</v>
+      </c>
+      <c r="B176" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>179</v>
+      </c>
+      <c r="B177" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
a lot of admin pages
</commit_message>
<xml_diff>
--- a/docs/TimeSheet.xlsx
+++ b/docs/TimeSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\workplace\lsevin\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC38802-6E75-467D-B0B8-4F16F51FFD84}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58C5E5D6-7889-4F10-9021-BB4EFC577497}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3C67C6F1-DCD5-4F32-8E1E-2D0F4630EB6C}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="212">
   <si>
     <t xml:space="preserve">عنوان </t>
   </si>
@@ -607,13 +607,73 @@
   </si>
   <si>
     <t>my bookings</t>
+  </si>
+  <si>
+    <t>booking-drafts</t>
+  </si>
+  <si>
+    <t>bookings</t>
+  </si>
+  <si>
+    <t>customers</t>
+  </si>
+  <si>
+    <t>identity-users</t>
+  </si>
+  <si>
+    <t>loyalty</t>
+  </si>
+  <si>
+    <t>marketing</t>
+  </si>
+  <si>
+    <t>/payments</t>
+  </si>
+  <si>
+    <t>platform-data</t>
+  </si>
+  <si>
+    <t>wallet-payment-intents</t>
+  </si>
+  <si>
+    <t>wallet-transactions</t>
+  </si>
+  <si>
+    <t>Service Definitions</t>
+  </si>
+  <si>
+    <t>Provider Services</t>
+  </si>
+  <si>
+    <t>Service Add-ons</t>
+  </si>
+  <si>
+    <t>Service Gallery</t>
+  </si>
+  <si>
+    <t>Service Upload File Requirements</t>
+  </si>
+  <si>
+    <t>Service FAQs</t>
+  </si>
+  <si>
+    <t>Service Included Items</t>
+  </si>
+  <si>
+    <t>Service Process Steps</t>
+  </si>
+  <si>
+    <t>Service Definition Add-on Provider Types</t>
+  </si>
+  <si>
+    <t xml:space="preserve">provider details </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -632,6 +692,14 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -672,7 +740,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -685,6 +753,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -999,10 +1068,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5151749-D98A-4C10-BD15-AFBB1EC4BCB9}">
-  <dimension ref="A1:F177"/>
+  <dimension ref="A1:F198"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" customWidth="1"/>
     <col min="3" max="3" width="43.140625" customWidth="1"/>
     <col min="4" max="4" width="25.140625" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
@@ -2174,6 +2243,171 @@
         <v>191</v>
       </c>
     </row>
+    <row r="178" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>179</v>
+      </c>
+      <c r="B179" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>179</v>
+      </c>
+      <c r="B180" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>179</v>
+      </c>
+      <c r="B181" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>179</v>
+      </c>
+      <c r="B182" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>179</v>
+      </c>
+      <c r="B183" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>179</v>
+      </c>
+      <c r="B184" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>179</v>
+      </c>
+      <c r="B185" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>179</v>
+      </c>
+      <c r="B186" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>179</v>
+      </c>
+      <c r="B187" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>179</v>
+      </c>
+      <c r="B188" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>179</v>
+      </c>
+      <c r="B189" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>179</v>
+      </c>
+      <c r="B190" s="8" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>179</v>
+      </c>
+      <c r="B191" s="8" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>179</v>
+      </c>
+      <c r="B192" s="8" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>179</v>
+      </c>
+      <c r="B193" s="8" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>179</v>
+      </c>
+      <c r="B194" s="8" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>179</v>
+      </c>
+      <c r="B195" s="8" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>179</v>
+      </c>
+      <c r="B196" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>179</v>
+      </c>
+      <c r="B197" s="8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>179</v>
+      </c>
+      <c r="B198" s="8" t="s">
+        <v>211</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>